<commit_message>
chore: update summary Excel with off-platform cash income section
</commit_message>
<xml_diff>
--- a/vault/thoughts/projects/arenda-kvartir-tashkent/files/Свод_Самарканд_доход_расход_окупаемость.xlsx
+++ b/vault/thoughts/projects/arenda-kvartir-tashkent/files/Свод_Самарканд_доход_расход_окупаемость.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Сводка" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Чёрная касса" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="По объектам" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Окупаемость" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Нал вне платформ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="По объектам" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Окупаемость" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,7 +57,7 @@
       <color rgb="00A3402F"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDE6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6ECD9"/>
       </patternFill>
     </fill>
     <fill>
@@ -110,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,10 +127,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -625,145 +633,232 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>1.5. + НАЛ ВНЕ ПЛАТФОРМ ('сарафанное радио', заявлено партнёром письменно)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Это НЕ подтверждено ни одной платформой — только собственноручная запись партнёра. Показано отдельно, не смешано с официальным доходом выше.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Источник</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Ночей</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Доход $</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>'Сарафанное радио' (3 записи, все — White Pearl)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Подробный список по дням — на листе 'Нал вне платформ'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>11 других строк с пометкой 'наличные' в таблице партнёра — это Booking-брони, оплаченные наличными на месте; они уже учтены в официальном доходе выше, отдельно не добавлены во избежание задвоения.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>2. РАСХОДЫ ПО ТАБЛИЦЕ ПАРТНЁРА (январь–июнь 2026)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Сумма, сум</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>≈ $, по курсу выше</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Все расходы (аренда, уборка, быт и т.д.)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B23" s="6" t="n">
         <v>143845780</v>
       </c>
-      <c r="C16" s="6">
-        <f>B16/$B$5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="C23" s="6">
+        <f>B23/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  из них разовые ('вложения'/обустройство)</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B24" s="6" t="n">
         <v>38122800</v>
       </c>
-      <c r="C17" s="6">
-        <f>B17/$B$5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="C24" s="6">
+        <f>B24/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  из них периодические (аренда, коммуналка, уборка)</t>
         </is>
       </c>
-      <c r="B18" s="6">
-        <f>B16-B17</f>
-        <v/>
-      </c>
-      <c r="C18" s="6">
-        <f>B18/$B$5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>3. ИТОГ: ПРИБЫЛЬ / УБЫТОК ПО ОФИЦИАЛЬНЫМ ДАННЫМ</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Официальный доход $</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B25" s="6">
+        <f>B23-B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="6">
+        <f>B25/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>3. ИТОГ: ПРИБЫЛЬ / УБЫТОК — ДВА СЦЕНАРИЯ</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Сценарий</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Доход $</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Расходы $ (по курсу)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Прибыль(+) / Убыток(-) $</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8">
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Только официально подтверждённое (Booking+Airbnb)</t>
+        </is>
+      </c>
+      <c r="B29" s="9">
         <f>D12</f>
         <v/>
       </c>
-      <c r="B22" s="8">
-        <f>C16</f>
-        <v/>
-      </c>
-      <c r="C22" s="8">
-        <f>A22-B22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Отрицательное число = по проверяемым платформенным деньгам бизнес пока НЕ окупается и не в плюсе.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Это не значит, что реальных денег нет — см. лист 'Чёрная касса': минимум $1 574 подтверждённого дохода одной из квартир записано партнёром как $0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="C29" s="9">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="D29" s="10">
+        <f>B29-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>+ нал, заявленный партнёром письменно ('сарафанное радио')</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>D12+C17</f>
+        <v/>
+      </c>
+      <c r="C30" s="9">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="D30" s="10">
+        <f>B30-C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Оба варианта — минус. $260 погоды не делают на фоне убытка в тысячи долларов.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Отдельно от обоих сценариев: минимум $1 574 подтверждённого Booking.com дохода Black Pearl записано партнёром как $0 — это не 'нал', это платформенные деньги, которые официально уже есть в строке 'Booking.com' выше, но по ним не ясно, кто их получил. Подробности — лист 'Чёрная касса'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>4. ГЛАВНАЯ НАХОДКА</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>В таблице партнёра квартира 'Black Pearl' (= Spacious apartment / Registan) три месяца подряд — апрель, май, июнь — показывает официально подтверждённые брони Booking.com, а записанный доход по ним каждый месяц: 0 сум / $0.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>'White Pearl' (= квартира у аэропорта) за те же месяцы отражена в этой же таблице подробно и построчно, вплоть до Airbnb-выплат в долларах.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Подробности и прямая сверка с датами Booking.com — на листе 'Чёрная касса'.</t>
         </is>
@@ -832,59 +927,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Апрель</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="9" t="n">
         <v>863.01</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Май</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="9" t="n">
         <v>483.59</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Июнь</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="9" t="n">
         <v>227.8</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -918,7 +1013,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Минимум $1,574.40 — это НЕ предположение, это официальная сумма из выгрузки Booking.com за подтверждённые (OK) брони этой квартиры за апрель-июнь.</t>
         </is>
@@ -972,6 +1067,408 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>'Сарафанное радио' — весь нал, заявленный партнёром письменно, по дням</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ни одна из этих сумм не подтверждена платформой — это только собственноручная запись партнёра в его же таблице.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Заезд</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Выезд</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Ночей</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Сумма $</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Квартира</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Способ оплаты (как указал партнёр)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>03.04</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>05.04</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>White Pearl</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>наличные, без комиссии</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>24.06</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>26.06</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>White Pearl</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>наличные, без комиссии</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>26.06</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>29.06</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>White Pearl</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>наличные, без комиссии</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr"/>
+      <c r="C8" s="7">
+        <f>SUM(C5:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>SUM(D5:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Для справки: остальные 11 строк 'наличные' в таблице партнёра</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Это Booking-брони, за которые гость заплатил наличными на месте, а не через сайт. Даты этих 11 броней уже присутствуют в официальной выгрузке Booking.com и уже включены в 'Официальный доход' на листе 'Сводка' — здесь не задвоены.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Заезд</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Выезд</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>09.05</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>10.05</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>10.05</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>13.05</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>18.05</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>19.05</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>22.05</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>23.05</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>23.05</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>24.05</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>25.05</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>27.05</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>27.05</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>29.05</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>06.06</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>07.06</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>12.06</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>13.06</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>14.06</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>15.06</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>18.06</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>21.06</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>уже в официальном доходе Booking.com — не добавлять повторно</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Отдельная пометка про 'битые' ячейки</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>В той же таблице (лист 'Доходы', столбцы правее) есть блок с числами вроде 635 999 в графе 'Кол-во ночей' — это физически невозможно (636 тысяч ночей). Похоже на сломанную/протянутую формулу, а не на реальные данные. В расчёт не включено — стоит спросить у партнёра, что это такое.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1034,17 +1531,17 @@
           <t>Black Pearl (Spacious/Registan)</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="9" t="n">
         <v>3534.24</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="9" t="n">
         <v>88005130</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <f>C5/Сводка!$B$5</f>
         <v/>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="9">
         <f>B5-D5</f>
         <v/>
       </c>
@@ -1055,17 +1552,17 @@
           <t>White Pearl (у аэропорта)</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="9" t="n">
         <v>2465.37</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="9" t="n">
         <v>46577650</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <f>C6/Сводка!$B$5</f>
         <v/>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <f>B6-D6</f>
         <v/>
       </c>
@@ -1133,7 +1630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>